<commit_message>
🎨 feat: match history shows per-game rating changes with role column
Each game on the match-history page now renders as a last-game-style
table (rank, player, role, result, rating, change) instead of an
alignment-only card. Role column shows Mafia/Cop/Medic/Vigilante/Town.

backend/main.py get_match_history returns the same per-player shape as
get_last_game, including rate_change, old_rating, new_rating. The
Alignment column in MatchHistory already stores the literal role for
games recorded through record_game, so no schema migration is needed.

ego-mafia/data.json is regenerated by process_games.py with a per-game
players[] list. The history-row schema now stores the literal role
(Cop/Medic/Vigilante) instead of collapsing town members to "Town".
bootstrap_sheet.py mirrors this change for the live sheet.

ego-mafia/match-history.css is removed — the page reuses root style.css
.last-game styling with a small match-history.css overlay.
</commit_message>
<xml_diff>
--- a/ego_mafia/match_results.xlsx
+++ b/ego_mafia/match_results.xlsx
@@ -1106,7 +1106,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Town</t>
+          <t>Vigilante</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Town</t>
+          <t>Medic</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Town</t>
+          <t>Cop</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Town</t>
+          <t>Vigilante</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Town</t>
+          <t>Medic</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Town</t>
+          <t>Cop</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">

</xml_diff>

<commit_message>
🔧 config: tune ego-mafia TrueSkill priors to ~53% mafia winrate
Ghost-mu gap reduced from 1.85 → 0.37 (mafia 25.7→24.96,
town 23.85→24.59) and beta reduced 5.5 → 5.0. Targets a ~53%
prior mafia winrate at default sigma, vs ~65% under the old
parameters. Better reflects observed elo-lobby outcomes (~50%
over 108 games). Midpoint preserved at 24.775 so absolute
rating scale stays comparable to the casual backend.

match_results.xlsx and data.json regenerated from games_input.csv
with the new parameters.
</commit_message>
<xml_diff>
--- a/ego_mafia/match_results.xlsx
+++ b/ego_mafia/match_results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="MatchRatings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="MatchHistory" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MatchRatings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MatchHistory" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,13 +446,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>27.20136491482106</v>
+        <v>27.25829894295319</v>
       </c>
       <c r="C2" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="D2" t="n">
-        <v>1014</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="3">
@@ -462,13 +462,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>27.20136491482106</v>
+        <v>27.25829894295319</v>
       </c>
       <c r="C3" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="D3" t="n">
-        <v>1014</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="4">
@@ -478,13 +478,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26.43032996689729</v>
+        <v>26.2164448820499</v>
       </c>
       <c r="C4" t="n">
-        <v>8.2543528944042</v>
+        <v>8.253863000563229</v>
       </c>
       <c r="D4" t="n">
-        <v>955</v>
+        <v>941</v>
       </c>
     </row>
     <row r="5">
@@ -494,13 +494,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>26.43032996689729</v>
+        <v>26.2164448820499</v>
       </c>
       <c r="C5" t="n">
-        <v>8.2543528944042</v>
+        <v>8.253863000563229</v>
       </c>
       <c r="D5" t="n">
-        <v>955</v>
+        <v>941</v>
       </c>
     </row>
     <row r="6">
@@ -510,13 +510,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="C6" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="D6" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
     </row>
     <row r="7">
@@ -526,13 +526,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="C7" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="D7" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
     </row>
     <row r="8">
@@ -542,13 +542,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="C8" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="D8" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
     </row>
     <row r="9">
@@ -558,13 +558,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="C9" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="D9" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
     </row>
     <row r="10">
@@ -574,13 +574,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="C10" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="D10" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
     </row>
     <row r="11">
@@ -590,13 +590,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="C11" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="D11" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
     </row>
     <row r="12">
@@ -606,13 +606,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>24.38215434625663</v>
+        <v>24.86866117825723</v>
       </c>
       <c r="C12" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="D12" t="n">
-        <v>822</v>
+        <v>857</v>
       </c>
     </row>
     <row r="13">
@@ -622,13 +622,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="C13" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="D13" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
     </row>
     <row r="14">
@@ -638,13 +638,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="C14" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="D14" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
     </row>
     <row r="15">
@@ -654,13 +654,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>22.79863508517894</v>
+        <v>22.7417010570468</v>
       </c>
       <c r="C15" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="D15" t="n">
-        <v>714</v>
+        <v>712</v>
       </c>
     </row>
     <row r="16">
@@ -670,13 +670,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>22.79863508517894</v>
+        <v>22.7417010570468</v>
       </c>
       <c r="C16" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="D16" t="n">
-        <v>714</v>
+        <v>712</v>
       </c>
     </row>
   </sheetData>
@@ -828,22 +828,22 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="F4" t="n">
         <v>25</v>
       </c>
       <c r="G4" t="n">
-        <v>26.43032996689729</v>
+        <v>26.2164448820499</v>
       </c>
       <c r="H4" t="n">
-        <v>8.2543528944042</v>
+        <v>8.253863000563229</v>
       </c>
       <c r="I4" t="n">
         <v>850</v>
       </c>
       <c r="J4" t="n">
-        <v>955</v>
+        <v>941</v>
       </c>
       <c r="K4" t="n">
         <v>8.333333333333334</v>
@@ -869,25 +869,25 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="F5" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="G5" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="H5" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="I5" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="J5" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
       <c r="K5" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
     </row>
     <row r="6">
@@ -910,25 +910,25 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="F6" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="G6" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="H6" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="I6" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="J6" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
       <c r="K6" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
     </row>
     <row r="7">
@@ -951,25 +951,25 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="F7" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="G7" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="H7" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="I7" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="J7" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
       <c r="K7" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
     </row>
     <row r="8">
@@ -992,25 +992,25 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="F8" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="G8" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="H8" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="I8" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="J8" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
       <c r="K8" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
     </row>
     <row r="9">
@@ -1033,25 +1033,25 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="F9" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="G9" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="H9" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="I9" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="J9" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
       <c r="K9" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
     </row>
     <row r="10">
@@ -1074,25 +1074,25 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="F10" t="n">
-        <v>25.79175963053884</v>
+        <v>26.06348006060521</v>
       </c>
       <c r="G10" t="n">
-        <v>27.20136491482106</v>
+        <v>27.25829894295319</v>
       </c>
       <c r="H10" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="I10" t="n">
-        <v>910</v>
+        <v>930</v>
       </c>
       <c r="J10" t="n">
-        <v>1014</v>
+        <v>1019</v>
       </c>
       <c r="K10" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
     </row>
     <row r="11">
@@ -1115,22 +1115,22 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="F11" t="n">
         <v>25</v>
       </c>
       <c r="G11" t="n">
-        <v>26.43032996689729</v>
+        <v>26.2164448820499</v>
       </c>
       <c r="H11" t="n">
-        <v>8.2543528944042</v>
+        <v>8.253863000563229</v>
       </c>
       <c r="I11" t="n">
         <v>850</v>
       </c>
       <c r="J11" t="n">
-        <v>955</v>
+        <v>941</v>
       </c>
       <c r="K11" t="n">
         <v>8.333333333333334</v>
@@ -1156,25 +1156,25 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="F12" t="n">
-        <v>25.79175963053884</v>
+        <v>26.06348006060521</v>
       </c>
       <c r="G12" t="n">
-        <v>27.20136491482106</v>
+        <v>27.25829894295319</v>
       </c>
       <c r="H12" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="I12" t="n">
-        <v>910</v>
+        <v>930</v>
       </c>
       <c r="J12" t="n">
-        <v>1014</v>
+        <v>1019</v>
       </c>
       <c r="K12" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
     </row>
     <row r="13">
@@ -1197,25 +1197,25 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="F13" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="G13" t="n">
-        <v>25.61784565374338</v>
+        <v>25.13133882174276</v>
       </c>
       <c r="H13" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="I13" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="J13" t="n">
-        <v>906</v>
+        <v>874</v>
       </c>
       <c r="K13" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
     </row>
     <row r="14">
@@ -1238,25 +1238,25 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>-88</v>
+        <v>-73</v>
       </c>
       <c r="F14" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="G14" t="n">
-        <v>22.79863508517894</v>
+        <v>22.7417010570468</v>
       </c>
       <c r="H14" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="I14" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="J14" t="n">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="K14" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
     </row>
     <row r="15">
@@ -1279,25 +1279,25 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>-88</v>
+        <v>-73</v>
       </c>
       <c r="F15" t="n">
-        <v>25.79175963053884</v>
+        <v>26.06348006060521</v>
       </c>
       <c r="G15" t="n">
-        <v>24.38215434625663</v>
+        <v>24.86866117825723</v>
       </c>
       <c r="H15" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="I15" t="n">
-        <v>910</v>
+        <v>930</v>
       </c>
       <c r="J15" t="n">
-        <v>822</v>
+        <v>857</v>
       </c>
       <c r="K15" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
     </row>
     <row r="16">
@@ -1320,25 +1320,25 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>-88</v>
+        <v>-73</v>
       </c>
       <c r="F16" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="G16" t="n">
-        <v>22.79863508517894</v>
+        <v>22.7417010570468</v>
       </c>
       <c r="H16" t="n">
-        <v>8.195484338342377</v>
+        <v>8.181582751422322</v>
       </c>
       <c r="I16" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="J16" t="n">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="K16" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
     </row>
     <row r="17">
@@ -1419,22 +1419,22 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>-48</v>
+        <v>-65</v>
       </c>
       <c r="F19" t="n">
         <v>25</v>
       </c>
       <c r="G19" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="H19" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I19" t="n">
         <v>850</v>
       </c>
       <c r="J19" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="K19" t="n">
         <v>8.333333333333334</v>
@@ -1460,22 +1460,22 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>-48</v>
+        <v>-65</v>
       </c>
       <c r="F20" t="n">
         <v>25</v>
       </c>
       <c r="G20" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="H20" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I20" t="n">
         <v>850</v>
       </c>
       <c r="J20" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="K20" t="n">
         <v>8.333333333333334</v>
@@ -1501,22 +1501,22 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>-48</v>
+        <v>-65</v>
       </c>
       <c r="F21" t="n">
         <v>25</v>
       </c>
       <c r="G21" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="H21" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I21" t="n">
         <v>850</v>
       </c>
       <c r="J21" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="K21" t="n">
         <v>8.333333333333334</v>
@@ -1542,22 +1542,22 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>-48</v>
+        <v>-65</v>
       </c>
       <c r="F22" t="n">
         <v>25</v>
       </c>
       <c r="G22" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="H22" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I22" t="n">
         <v>850</v>
       </c>
       <c r="J22" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="K22" t="n">
         <v>8.333333333333334</v>
@@ -1583,22 +1583,22 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>-48</v>
+        <v>-65</v>
       </c>
       <c r="F23" t="n">
         <v>25</v>
       </c>
       <c r="G23" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="H23" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I23" t="n">
         <v>850</v>
       </c>
       <c r="J23" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="K23" t="n">
         <v>8.333333333333334</v>
@@ -1624,22 +1624,22 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>-48</v>
+        <v>-65</v>
       </c>
       <c r="F24" t="n">
         <v>25</v>
       </c>
       <c r="G24" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="H24" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I24" t="n">
         <v>850</v>
       </c>
       <c r="J24" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="K24" t="n">
         <v>8.333333333333334</v>
@@ -1665,22 +1665,22 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>-48</v>
+        <v>-65</v>
       </c>
       <c r="F25" t="n">
         <v>25</v>
       </c>
       <c r="G25" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="H25" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I25" t="n">
         <v>850</v>
       </c>
       <c r="J25" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="K25" t="n">
         <v>8.333333333333334</v>
@@ -1706,22 +1706,22 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>-48</v>
+        <v>-65</v>
       </c>
       <c r="F26" t="n">
         <v>25</v>
       </c>
       <c r="G26" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="H26" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I26" t="n">
         <v>850</v>
       </c>
       <c r="J26" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="K26" t="n">
         <v>8.333333333333334</v>
@@ -1747,22 +1747,22 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>-48</v>
+        <v>-65</v>
       </c>
       <c r="F27" t="n">
         <v>25</v>
       </c>
       <c r="G27" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="H27" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I27" t="n">
         <v>850</v>
       </c>
       <c r="J27" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="K27" t="n">
         <v>8.333333333333334</v>
@@ -1788,22 +1788,22 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>-48</v>
+        <v>-65</v>
       </c>
       <c r="F28" t="n">
         <v>25</v>
       </c>
       <c r="G28" t="n">
-        <v>24.20824036946116</v>
+        <v>23.93651993939477</v>
       </c>
       <c r="H28" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I28" t="n">
         <v>850</v>
       </c>
       <c r="J28" t="n">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="K28" t="n">
         <v>8.333333333333334</v>
@@ -1829,22 +1829,22 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F29" t="n">
         <v>25</v>
       </c>
       <c r="G29" t="n">
-        <v>25.79175963053884</v>
+        <v>26.06348006060521</v>
       </c>
       <c r="H29" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I29" t="n">
         <v>850</v>
       </c>
       <c r="J29" t="n">
-        <v>910</v>
+        <v>930</v>
       </c>
       <c r="K29" t="n">
         <v>8.333333333333334</v>
@@ -1870,22 +1870,22 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F30" t="n">
         <v>25</v>
       </c>
       <c r="G30" t="n">
-        <v>25.79175963053884</v>
+        <v>26.06348006060521</v>
       </c>
       <c r="H30" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I30" t="n">
         <v>850</v>
       </c>
       <c r="J30" t="n">
-        <v>910</v>
+        <v>930</v>
       </c>
       <c r="K30" t="n">
         <v>8.333333333333334</v>
@@ -1911,22 +1911,22 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F31" t="n">
         <v>25</v>
       </c>
       <c r="G31" t="n">
-        <v>25.79175963053884</v>
+        <v>26.06348006060521</v>
       </c>
       <c r="H31" t="n">
-        <v>8.272731611951896</v>
+        <v>8.258915237453891</v>
       </c>
       <c r="I31" t="n">
         <v>850</v>
       </c>
       <c r="J31" t="n">
-        <v>910</v>
+        <v>930</v>
       </c>
       <c r="K31" t="n">
         <v>8.333333333333334</v>

</xml_diff>